<commit_message>
corrigiendo la generacion de archivos
</commit_message>
<xml_diff>
--- a/public/forms/02.xlsx
+++ b/public/forms/02.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/689d1a227c82b3ba/Documents/cuenta cobro/enero/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\victor\proyectos\viva\vivapay\public\forms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="117" documentId="8_{819D694B-DD82-427F-A74E-36A49FE0B8D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD0C3B3B-EF96-412D-A664-5129936833E1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D0EA9B0-7B63-4E63-BA1B-171929DECBEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="3696" yWindow="2844" windowWidth="17280" windowHeight="8880" tabRatio="324" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="324" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GFR-FO-17 " sheetId="13" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="201">
   <si>
     <t>INFORME DE EJECUCIÓN CONTRACTUTAL
 PRESTADORES DE SERVICIOS PERSONALES</t>
@@ -724,77 +724,10 @@
     <t>Cuando el pago esté asociado a varios rubros presupuestales y/o centros de costos debe estar debidamente discriminado el valor a afectar por cada uno.</t>
   </si>
   <si>
-    <t>Victor Manuel Cordoba Cordoba</t>
-  </si>
-  <si>
-    <t>CPS-99-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WILLMAR DARIO AGUDELO DAVILA </t>
-  </si>
-  <si>
-    <t>6 MESES</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 2.3.2.02.02.008.20.01</t>
-  </si>
-  <si>
-    <t>119 del 20/01/2026</t>
-  </si>
-  <si>
-    <t>291 del  28/01/2026</t>
-  </si>
-  <si>
-    <t>02VIVA001</t>
-  </si>
-  <si>
     <t>NO (  X)</t>
   </si>
   <si>
     <t>SI ( X )</t>
-  </si>
-  <si>
-    <t>1.  Apoyar el desarrollo de aplicativos y sistemas de software para el funcionamiento de los 
-procesos y operaciones de la Empresa de Vivienda de Antioquia – VIVA.</t>
-  </si>
-  <si>
-    <t>2. Apoyar en las acciones operativas necesarias para el funcionamiento del área de 
-Tecnologías de la Información (TI)</t>
-  </si>
-  <si>
-    <t>3. Apoyar en la elaboración de informes de seguimiento necesarios requeridos por la 
-coordinación y dirección administrativa y financiera referentes al funcionamiento del área 
-de Tecnologías de la Información (TI)</t>
-  </si>
-  <si>
-    <t>4. Apoyar en la construcción de aplicativos basados en LowCode y código nativo para 
-gestionar procesos entre las distintas direcciones, jefaturas y la gerencia de la Empresa 
-de Vivienda de Antioquia -VIVA.</t>
-  </si>
-  <si>
-    <t>Desplegar VIVAMAT con dominio de pruebacompleted</t>
-  </si>
-  <si>
-    <t>Manejo Integral de Estados del Pedidocompleted</t>
-  </si>
-  <si>
-    <t>REESTRUCTURAR LA Dbcompleted</t>
-  </si>
-  <si>
-    <t>Preparar codigo para productioncompleted</t>
-  </si>
-  <si>
-    <t>https://github.com/Victordi10/viva-mat.git</t>
-  </si>
-  <si>
-    <t>https://github.com/Victordi10/gogo-viva.git</t>
-  </si>
-  <si>
-    <t>5,Apoyar en la implementación de nuevas tecnologías para el control y funcionamiento de
-la Empresa de Vivienda de Antioquia – VIVA.</t>
-  </si>
-  <si>
-    <t>PRESTACION DE SERVICIOS COMO APOYO A LOS DIFERENTES PROCESOS DE LA DIRECCION DMINISTRATIVA Y FINANCIERA DE LA EMPRESA DE VIVIENDA DE ANTIOQUIA –VIVA</t>
   </si>
   <si>
     <t>CIENTO DOCE MIL DOCIENTOS TREINTA Y CINCO PESOS M/L</t>
@@ -2101,6 +2034,283 @@
     <xf numFmtId="165" fontId="22" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="22" fillId="5" borderId="11" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="22" fillId="5" borderId="4" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="6" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="7" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="8" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="6" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="24" fillId="4" borderId="6" xfId="3" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="24" fillId="4" borderId="8" xfId="3" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="24" fillId="4" borderId="9" xfId="3" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="14" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="8" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="8" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="23" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="8" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="4" borderId="9" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="13" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="14" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="9" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="6" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="7" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="8" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -2109,18 +2319,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="9" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="6" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="7" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="8" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -2129,271 +2327,6 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="23" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="8" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="13" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="14" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="6" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="7" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="8" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="6" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="24" fillId="4" borderId="9" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="17" fontId="24" fillId="4" borderId="6" xfId="3" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="24" fillId="4" borderId="8" xfId="3" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="24" fillId="4" borderId="9" xfId="3" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="14" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="24" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="8" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="8" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="22" fillId="5" borderId="11" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="43" fontId="22" fillId="5" borderId="4" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="7" borderId="9" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2526,56 +2459,6 @@
         <a:xfrm>
           <a:off x="1636939" y="163286"/>
           <a:ext cx="2390775" cy="1259950"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>811867</xdr:colOff>
-      <xdr:row>121</xdr:row>
-      <xdr:rowOff>62109</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>818029</xdr:colOff>
-      <xdr:row>122</xdr:row>
-      <xdr:rowOff>352984</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DAF8B548-48E6-C5C4-31CA-EB4FCB6345F6}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2178985" y="28670727"/>
-          <a:ext cx="1037103" cy="470169"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2903,34 +2786,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="117.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="277" t="s">
+      <c r="A1" s="318" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="278"/>
-      <c r="C1" s="278"/>
-      <c r="D1" s="278"/>
-      <c r="E1" s="278"/>
-      <c r="F1" s="278"/>
-      <c r="G1" s="278"/>
-      <c r="H1" s="278"/>
-      <c r="I1" s="278"/>
-      <c r="J1" s="278"/>
-      <c r="K1" s="279"/>
+      <c r="B1" s="319"/>
+      <c r="C1" s="319"/>
+      <c r="D1" s="319"/>
+      <c r="E1" s="319"/>
+      <c r="F1" s="319"/>
+      <c r="G1" s="319"/>
+      <c r="H1" s="319"/>
+      <c r="I1" s="319"/>
+      <c r="J1" s="319"/>
+      <c r="K1" s="320"/>
     </row>
     <row r="2" spans="1:31" s="15" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="257" t="s">
+      <c r="A2" s="321" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="257"/>
-      <c r="C2" s="257"/>
-      <c r="D2" s="257"/>
-      <c r="E2" s="257"/>
-      <c r="F2" s="257"/>
-      <c r="G2" s="257"/>
-      <c r="H2" s="257"/>
-      <c r="I2" s="257"/>
-      <c r="J2" s="257"/>
-      <c r="K2" s="257"/>
+      <c r="B2" s="321"/>
+      <c r="C2" s="321"/>
+      <c r="D2" s="321"/>
+      <c r="E2" s="321"/>
+      <c r="F2" s="321"/>
+      <c r="G2" s="321"/>
+      <c r="H2" s="321"/>
+      <c r="I2" s="321"/>
+      <c r="J2" s="321"/>
+      <c r="K2" s="321"/>
       <c r="AC2" s="15" t="s">
         <v>2</v>
       </c>
@@ -2959,14 +2842,12 @@
       </c>
     </row>
     <row r="4" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="304" t="s">
+      <c r="A4" s="277" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="305"/>
-      <c r="C4" s="286" t="s">
-        <v>198</v>
-      </c>
-      <c r="D4" s="287"/>
+      <c r="B4" s="278"/>
+      <c r="C4" s="279"/>
+      <c r="D4" s="280"/>
       <c r="E4" s="183" t="s">
         <v>7</v>
       </c>
@@ -2976,10 +2857,8 @@
       <c r="G4" s="185" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="286">
-        <v>1000191780</v>
-      </c>
-      <c r="I4" s="287"/>
+      <c r="H4" s="279"/>
+      <c r="I4" s="280"/>
       <c r="J4" s="184"/>
       <c r="K4" s="92"/>
       <c r="AC4" s="2" t="s">
@@ -3009,23 +2888,19 @@
       </c>
     </row>
     <row r="6" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="304" t="s">
+      <c r="A6" s="277" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="305"/>
-      <c r="C6" s="306" t="s">
-        <v>199</v>
-      </c>
-      <c r="D6" s="307"/>
-      <c r="E6" s="308" t="s">
+      <c r="B6" s="278"/>
+      <c r="C6" s="281"/>
+      <c r="D6" s="282"/>
+      <c r="E6" s="283" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="309"/>
-      <c r="G6" s="310" t="s">
-        <v>11</v>
-      </c>
-      <c r="H6" s="310"/>
-      <c r="I6" s="310"/>
+      <c r="F6" s="284"/>
+      <c r="G6" s="285"/>
+      <c r="H6" s="285"/>
+      <c r="I6" s="285"/>
       <c r="J6" s="184"/>
       <c r="K6" s="92"/>
       <c r="AE6" s="2" t="s">
@@ -3053,19 +2928,15 @@
         <v>18</v>
       </c>
       <c r="B8" s="184"/>
-      <c r="C8" s="311" t="s">
-        <v>200</v>
-      </c>
-      <c r="D8" s="270"/>
-      <c r="E8" s="312"/>
+      <c r="C8" s="286"/>
+      <c r="D8" s="287"/>
+      <c r="E8" s="288"/>
       <c r="F8" s="184"/>
       <c r="G8" s="185" t="s">
         <v>9</v>
       </c>
-      <c r="H8" s="286">
-        <v>98663128</v>
-      </c>
-      <c r="I8" s="287"/>
+      <c r="H8" s="279"/>
+      <c r="I8" s="280"/>
       <c r="J8" s="187"/>
       <c r="K8" s="94"/>
       <c r="AE8" s="2" t="s">
@@ -3089,69 +2960,67 @@
       </c>
     </row>
     <row r="10" spans="1:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="297" t="s">
+      <c r="A10" s="334" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="271" t="s">
-        <v>219</v>
-      </c>
-      <c r="C10" s="272"/>
-      <c r="D10" s="272"/>
-      <c r="E10" s="272"/>
-      <c r="F10" s="272"/>
-      <c r="G10" s="272"/>
-      <c r="H10" s="272"/>
-      <c r="I10" s="272"/>
-      <c r="J10" s="272"/>
-      <c r="K10" s="273"/>
+      <c r="B10" s="312"/>
+      <c r="C10" s="313"/>
+      <c r="D10" s="313"/>
+      <c r="E10" s="313"/>
+      <c r="F10" s="313"/>
+      <c r="G10" s="313"/>
+      <c r="H10" s="313"/>
+      <c r="I10" s="313"/>
+      <c r="J10" s="313"/>
+      <c r="K10" s="314"/>
       <c r="N10" s="5"/>
       <c r="AE10" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="298"/>
-      <c r="B11" s="274"/>
-      <c r="C11" s="275"/>
-      <c r="D11" s="275"/>
-      <c r="E11" s="275"/>
-      <c r="F11" s="275"/>
-      <c r="G11" s="275"/>
-      <c r="H11" s="275"/>
-      <c r="I11" s="275"/>
-      <c r="J11" s="275"/>
-      <c r="K11" s="276"/>
+      <c r="A11" s="335"/>
+      <c r="B11" s="315"/>
+      <c r="C11" s="316"/>
+      <c r="D11" s="316"/>
+      <c r="E11" s="316"/>
+      <c r="F11" s="316"/>
+      <c r="G11" s="316"/>
+      <c r="H11" s="316"/>
+      <c r="I11" s="316"/>
+      <c r="J11" s="316"/>
+      <c r="K11" s="317"/>
       <c r="N11" s="5"/>
       <c r="AE11" s="2" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A12" s="298"/>
-      <c r="B12" s="274"/>
-      <c r="C12" s="275"/>
-      <c r="D12" s="275"/>
-      <c r="E12" s="275"/>
-      <c r="F12" s="275"/>
-      <c r="G12" s="275"/>
-      <c r="H12" s="275"/>
-      <c r="I12" s="275"/>
-      <c r="J12" s="275"/>
-      <c r="K12" s="276"/>
+      <c r="A12" s="335"/>
+      <c r="B12" s="315"/>
+      <c r="C12" s="316"/>
+      <c r="D12" s="316"/>
+      <c r="E12" s="316"/>
+      <c r="F12" s="316"/>
+      <c r="G12" s="316"/>
+      <c r="H12" s="316"/>
+      <c r="I12" s="316"/>
+      <c r="J12" s="316"/>
+      <c r="K12" s="317"/>
       <c r="N12" s="5"/>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A13" s="299"/>
-      <c r="B13" s="274"/>
-      <c r="C13" s="275"/>
-      <c r="D13" s="275"/>
-      <c r="E13" s="275"/>
-      <c r="F13" s="275"/>
-      <c r="G13" s="275"/>
-      <c r="H13" s="275"/>
-      <c r="I13" s="275"/>
-      <c r="J13" s="275"/>
-      <c r="K13" s="276"/>
+      <c r="A13" s="336"/>
+      <c r="B13" s="315"/>
+      <c r="C13" s="316"/>
+      <c r="D13" s="316"/>
+      <c r="E13" s="316"/>
+      <c r="F13" s="316"/>
+      <c r="G13" s="316"/>
+      <c r="H13" s="316"/>
+      <c r="I13" s="316"/>
+      <c r="J13" s="316"/>
+      <c r="K13" s="317"/>
       <c r="N13" s="5"/>
     </row>
     <row r="14" spans="1:31" s="13" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.25">
@@ -3190,47 +3059,27 @@
       <c r="N14" s="14"/>
     </row>
     <row r="15" spans="1:31" s="11" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="326" t="s">
+      <c r="A15" s="255" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="327" t="s">
-        <v>201</v>
-      </c>
-      <c r="C15" s="322">
-        <v>46052</v>
-      </c>
-      <c r="D15" s="322">
-        <v>46232</v>
-      </c>
-      <c r="E15" s="101" t="s">
-        <v>2</v>
-      </c>
-      <c r="F15" s="102" t="s">
-        <v>202</v>
-      </c>
-      <c r="G15" s="102" t="s">
-        <v>203</v>
-      </c>
-      <c r="H15" s="103">
-        <v>20202426</v>
-      </c>
-      <c r="I15" s="102" t="s">
-        <v>204</v>
-      </c>
-      <c r="J15" s="103">
-        <v>20202426</v>
-      </c>
-      <c r="K15" s="103">
-        <v>20202426</v>
-      </c>
+      <c r="B15" s="256"/>
+      <c r="C15" s="298"/>
+      <c r="D15" s="298"/>
+      <c r="E15" s="101"/>
+      <c r="F15" s="102"/>
+      <c r="G15" s="102"/>
+      <c r="H15" s="103"/>
+      <c r="I15" s="102"/>
+      <c r="J15" s="103"/>
+      <c r="K15" s="103"/>
       <c r="L15" s="85"/>
       <c r="N15" s="83"/>
     </row>
     <row r="16" spans="1:31" s="11" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="326"/>
-      <c r="B16" s="328"/>
-      <c r="C16" s="323"/>
-      <c r="D16" s="323"/>
+      <c r="A16" s="255"/>
+      <c r="B16" s="257"/>
+      <c r="C16" s="299"/>
+      <c r="D16" s="299"/>
       <c r="E16" s="101"/>
       <c r="F16" s="102"/>
       <c r="G16" s="102"/>
@@ -3360,16 +3209,13 @@
       <c r="D23" s="184"/>
       <c r="E23" s="184"/>
       <c r="F23" s="194"/>
-      <c r="G23" s="280" t="s">
+      <c r="G23" s="322" t="s">
         <v>40</v>
       </c>
-      <c r="H23" s="281"/>
-      <c r="I23" s="281"/>
-      <c r="J23" s="282"/>
-      <c r="K23" s="110">
-        <f>SUM(K15:K22)</f>
-        <v>20202426</v>
-      </c>
+      <c r="H23" s="323"/>
+      <c r="I23" s="323"/>
+      <c r="J23" s="324"/>
+      <c r="K23" s="110"/>
     </row>
     <row r="24" spans="1:26" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="238"/>
@@ -3385,19 +3231,19 @@
       <c r="K24" s="241"/>
     </row>
     <row r="25" spans="1:26" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="283" t="s">
+      <c r="A25" s="325" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="284"/>
-      <c r="C25" s="284"/>
-      <c r="D25" s="284"/>
-      <c r="E25" s="284"/>
-      <c r="F25" s="284"/>
-      <c r="G25" s="284"/>
-      <c r="H25" s="284"/>
-      <c r="I25" s="284"/>
-      <c r="J25" s="284"/>
-      <c r="K25" s="285"/>
+      <c r="B25" s="326"/>
+      <c r="C25" s="326"/>
+      <c r="D25" s="326"/>
+      <c r="E25" s="326"/>
+      <c r="F25" s="326"/>
+      <c r="G25" s="326"/>
+      <c r="H25" s="326"/>
+      <c r="I25" s="326"/>
+      <c r="J25" s="326"/>
+      <c r="K25" s="327"/>
       <c r="N25" s="5"/>
     </row>
     <row r="26" spans="1:26" ht="13.8" x14ac:dyDescent="0.25">
@@ -3421,9 +3267,7 @@
       <c r="D27" s="196" t="s">
         <v>42</v>
       </c>
-      <c r="E27" s="197">
-        <v>1</v>
-      </c>
+      <c r="E27" s="197"/>
       <c r="F27" s="195"/>
       <c r="G27" s="195"/>
       <c r="H27" s="195"/>
@@ -3447,23 +3291,19 @@
       <c r="N28" s="5"/>
     </row>
     <row r="29" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="304" t="s">
+      <c r="A29" s="277" t="s">
         <v>43</v>
       </c>
-      <c r="B29" s="305"/>
-      <c r="C29" s="316">
-        <v>46052</v>
-      </c>
-      <c r="D29" s="316"/>
+      <c r="B29" s="278"/>
+      <c r="C29" s="292"/>
+      <c r="D29" s="292"/>
       <c r="E29" s="195"/>
       <c r="F29" s="183" t="s">
         <v>44</v>
       </c>
-      <c r="G29" s="316">
-        <v>46052</v>
-      </c>
-      <c r="H29" s="316"/>
-      <c r="I29" s="316"/>
+      <c r="G29" s="292"/>
+      <c r="H29" s="292"/>
+      <c r="I29" s="292"/>
       <c r="J29" s="195"/>
       <c r="K29" s="112"/>
       <c r="L29" s="11"/>
@@ -3485,23 +3325,20 @@
       <c r="Z30" s="6"/>
     </row>
     <row r="31" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="304" t="s">
+      <c r="A31" s="277" t="s">
         <v>45</v>
       </c>
-      <c r="B31" s="305"/>
-      <c r="C31" s="317">
+      <c r="B31" s="278"/>
+      <c r="C31" s="293">
         <v>112235</v>
       </c>
-      <c r="D31" s="317"/>
-      <c r="E31" s="317"/>
-      <c r="F31" s="317"/>
-      <c r="G31" s="317"/>
-      <c r="H31" s="317"/>
-      <c r="I31" s="317"/>
-      <c r="J31" s="253">
-        <f>K23/6</f>
-        <v>3367071</v>
-      </c>
+      <c r="D31" s="293"/>
+      <c r="E31" s="293"/>
+      <c r="F31" s="293"/>
+      <c r="G31" s="293"/>
+      <c r="H31" s="293"/>
+      <c r="I31" s="293"/>
+      <c r="J31" s="253"/>
       <c r="K31" s="112"/>
       <c r="Z31" s="6"/>
     </row>
@@ -3511,7 +3348,7 @@
       </c>
       <c r="B32" s="186"/>
       <c r="C32" s="201" t="s">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="D32" s="202"/>
       <c r="E32" s="201"/>
@@ -3540,12 +3377,12 @@
       <c r="Z33" s="6"/>
     </row>
     <row r="34" spans="1:73" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="318"/>
-      <c r="B34" s="319"/>
-      <c r="C34" s="319"/>
-      <c r="D34" s="319"/>
-      <c r="E34" s="319"/>
-      <c r="F34" s="319"/>
+      <c r="A34" s="294"/>
+      <c r="B34" s="295"/>
+      <c r="C34" s="295"/>
+      <c r="D34" s="295"/>
+      <c r="E34" s="295"/>
+      <c r="F34" s="295"/>
       <c r="G34" s="202"/>
       <c r="H34" s="202"/>
       <c r="I34" s="202"/>
@@ -3558,10 +3395,10 @@
       <c r="A35" s="93"/>
       <c r="B35" s="184"/>
       <c r="C35" s="184"/>
-      <c r="D35" s="313" t="s">
+      <c r="D35" s="289" t="s">
         <v>48</v>
       </c>
-      <c r="E35" s="313"/>
+      <c r="E35" s="289"/>
       <c r="F35" s="115" t="s">
         <v>49</v>
       </c>
@@ -3581,19 +3418,13 @@
       <c r="A36" s="93"/>
       <c r="B36" s="184"/>
       <c r="C36" s="184"/>
-      <c r="D36" s="324" t="s">
+      <c r="D36" s="303" t="s">
         <v>52</v>
       </c>
-      <c r="E36" s="325"/>
-      <c r="F36" s="116">
-        <v>83967169</v>
-      </c>
-      <c r="G36" s="116">
-        <v>83967169</v>
-      </c>
-      <c r="H36" s="116">
-        <v>83967169</v>
-      </c>
+      <c r="E36" s="304"/>
+      <c r="F36" s="116"/>
+      <c r="G36" s="116"/>
+      <c r="H36" s="116"/>
       <c r="I36" s="202"/>
       <c r="J36" s="202"/>
       <c r="K36" s="114"/>
@@ -3604,19 +3435,13 @@
       <c r="A37" s="93"/>
       <c r="B37" s="184"/>
       <c r="C37" s="184"/>
-      <c r="D37" s="320" t="s">
+      <c r="D37" s="296" t="s">
         <v>53</v>
       </c>
-      <c r="E37" s="321"/>
-      <c r="F37" s="117">
-        <v>58363.5</v>
-      </c>
-      <c r="G37" s="117">
-        <v>58363.5</v>
-      </c>
-      <c r="H37" s="117">
-        <v>58363.55</v>
-      </c>
+      <c r="E37" s="297"/>
+      <c r="F37" s="117"/>
+      <c r="G37" s="117"/>
+      <c r="H37" s="117"/>
       <c r="I37" s="202"/>
       <c r="J37" s="202"/>
       <c r="K37" s="114"/>
@@ -3630,19 +3455,13 @@
       <c r="A38" s="93"/>
       <c r="B38" s="184"/>
       <c r="C38" s="184"/>
-      <c r="D38" s="324" t="s">
+      <c r="D38" s="303" t="s">
         <v>54</v>
       </c>
-      <c r="E38" s="325"/>
-      <c r="F38" s="117">
-        <v>7300</v>
-      </c>
-      <c r="G38" s="117">
-        <v>9400</v>
-      </c>
-      <c r="H38" s="117">
-        <v>400</v>
-      </c>
+      <c r="E38" s="304"/>
+      <c r="F38" s="117"/>
+      <c r="G38" s="117"/>
+      <c r="H38" s="117"/>
       <c r="I38" s="202"/>
       <c r="J38" s="202"/>
       <c r="K38" s="114"/>
@@ -3656,22 +3475,13 @@
       <c r="A39" s="93"/>
       <c r="B39" s="184"/>
       <c r="C39" s="184"/>
-      <c r="D39" s="320" t="s">
+      <c r="D39" s="296" t="s">
         <v>55</v>
       </c>
-      <c r="E39" s="321"/>
-      <c r="F39" s="118">
-        <f>F37/$C$31</f>
-        <v>0.52001158283957771</v>
-      </c>
-      <c r="G39" s="118">
-        <f t="shared" ref="G39" si="0">G37/$C$31</f>
-        <v>0.52001158283957771</v>
-      </c>
-      <c r="H39" s="118">
-        <f>H37/$C$31</f>
-        <v>0.52001202833340765</v>
-      </c>
+      <c r="E39" s="297"/>
+      <c r="F39" s="118"/>
+      <c r="G39" s="118"/>
+      <c r="H39" s="118"/>
       <c r="I39" s="202"/>
       <c r="J39" s="202"/>
       <c r="K39" s="114"/>
@@ -3685,22 +3495,13 @@
       <c r="A40" s="93"/>
       <c r="B40" s="184"/>
       <c r="C40" s="184"/>
-      <c r="D40" s="320" t="s">
+      <c r="D40" s="296" t="s">
         <v>56</v>
       </c>
-      <c r="E40" s="321"/>
-      <c r="F40" s="119">
-        <f>F38/F37</f>
-        <v>0.12507817385866166</v>
-      </c>
-      <c r="G40" s="119">
-        <f>G38/G37</f>
-        <v>0.16105956633855065</v>
-      </c>
-      <c r="H40" s="119">
-        <f>H38/H37</f>
-        <v>6.8535926961262638E-3</v>
-      </c>
+      <c r="E40" s="297"/>
+      <c r="F40" s="119"/>
+      <c r="G40" s="119"/>
+      <c r="H40" s="119"/>
       <c r="I40" s="202"/>
       <c r="J40" s="202"/>
       <c r="K40" s="114"/>
@@ -3750,24 +3551,24 @@
     </row>
     <row r="43" spans="1:73" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="93"/>
-      <c r="B43" s="264" t="s">
+      <c r="B43" s="337" t="s">
         <v>58</v>
       </c>
-      <c r="C43" s="265"/>
-      <c r="D43" s="264" t="s">
+      <c r="C43" s="338"/>
+      <c r="D43" s="337" t="s">
         <v>59</v>
       </c>
-      <c r="E43" s="265"/>
+      <c r="E43" s="338"/>
       <c r="F43" s="122" t="s">
         <v>60</v>
       </c>
       <c r="G43" s="122" t="s">
         <v>61</v>
       </c>
-      <c r="H43" s="264" t="s">
+      <c r="H43" s="337" t="s">
         <v>62</v>
       </c>
-      <c r="I43" s="265"/>
+      <c r="I43" s="338"/>
       <c r="J43" s="122" t="s">
         <v>63</v>
       </c>
@@ -3779,28 +3580,15 @@
     </row>
     <row r="44" spans="1:73" s="15" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="205"/>
-      <c r="B44" s="255" t="s">
-        <v>203</v>
-      </c>
-      <c r="C44" s="256"/>
-      <c r="D44" s="255" t="s">
-        <v>204</v>
-      </c>
-      <c r="E44" s="256"/>
-      <c r="F44" s="102" t="s">
-        <v>202</v>
-      </c>
-      <c r="G44" s="101" t="s">
-        <v>2</v>
-      </c>
-      <c r="H44" s="2" t="s">
-        <v>205</v>
-      </c>
+      <c r="B44" s="339"/>
+      <c r="C44" s="340"/>
+      <c r="D44" s="339"/>
+      <c r="E44" s="340"/>
+      <c r="F44" s="102"/>
+      <c r="G44" s="101"/>
+      <c r="H44" s="2"/>
       <c r="I44" s="127"/>
-      <c r="J44" s="128">
-        <f>C31</f>
-        <v>112235</v>
-      </c>
+      <c r="J44" s="128"/>
       <c r="K44" s="123"/>
       <c r="L44" s="254"/>
       <c r="M44" s="254"/>
@@ -3814,10 +3602,10 @@
     </row>
     <row r="45" spans="1:73" s="15" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="205"/>
-      <c r="B45" s="255"/>
-      <c r="C45" s="256"/>
-      <c r="D45" s="255"/>
-      <c r="E45" s="256"/>
+      <c r="B45" s="339"/>
+      <c r="C45" s="340"/>
+      <c r="D45" s="339"/>
+      <c r="E45" s="340"/>
       <c r="F45" s="124"/>
       <c r="G45" s="125"/>
       <c r="H45" s="126"/>
@@ -3832,10 +3620,10 @@
     </row>
     <row r="46" spans="1:73" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="93"/>
-      <c r="B46" s="255"/>
-      <c r="C46" s="256"/>
-      <c r="D46" s="255"/>
-      <c r="E46" s="256"/>
+      <c r="B46" s="339"/>
+      <c r="C46" s="340"/>
+      <c r="D46" s="339"/>
+      <c r="E46" s="340"/>
       <c r="F46" s="124"/>
       <c r="G46" s="125"/>
       <c r="H46" s="126"/>
@@ -3849,10 +3637,10 @@
     </row>
     <row r="47" spans="1:73" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="93"/>
-      <c r="B47" s="255"/>
-      <c r="C47" s="256"/>
-      <c r="D47" s="255"/>
-      <c r="E47" s="256"/>
+      <c r="B47" s="339"/>
+      <c r="C47" s="340"/>
+      <c r="D47" s="339"/>
+      <c r="E47" s="340"/>
       <c r="F47" s="129"/>
       <c r="G47" s="130"/>
       <c r="H47" s="130"/>
@@ -3866,10 +3654,10 @@
     </row>
     <row r="48" spans="1:73" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="93"/>
-      <c r="B48" s="255"/>
-      <c r="C48" s="256"/>
-      <c r="D48" s="255"/>
-      <c r="E48" s="256"/>
+      <c r="B48" s="339"/>
+      <c r="C48" s="340"/>
+      <c r="D48" s="339"/>
+      <c r="E48" s="340"/>
       <c r="F48" s="129"/>
       <c r="G48" s="130"/>
       <c r="H48" s="130"/>
@@ -3883,10 +3671,10 @@
     </row>
     <row r="49" spans="1:73" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="93"/>
-      <c r="B49" s="255"/>
-      <c r="C49" s="256"/>
-      <c r="D49" s="255"/>
-      <c r="E49" s="256"/>
+      <c r="B49" s="339"/>
+      <c r="C49" s="340"/>
+      <c r="D49" s="339"/>
+      <c r="E49" s="340"/>
       <c r="F49" s="129"/>
       <c r="G49" s="130"/>
       <c r="H49" s="130"/>
@@ -3912,7 +3700,7 @@
       </c>
       <c r="J50" s="134">
         <f>SUM(J44:J49)</f>
-        <v>112235</v>
+        <v>0</v>
       </c>
       <c r="K50" s="114"/>
       <c r="Z50" s="6"/>
@@ -3984,10 +3772,7 @@
         <f>F53+G53</f>
         <v>0</v>
       </c>
-      <c r="I53" s="145">
-        <f>K23-H53</f>
-        <v>20202426</v>
-      </c>
+      <c r="I53" s="145"/>
       <c r="J53" s="212"/>
       <c r="K53" s="141"/>
       <c r="L53" s="11"/>
@@ -4008,13 +3793,10 @@
       <c r="F54" s="144"/>
       <c r="G54" s="144"/>
       <c r="H54" s="144">
-        <f t="shared" ref="H54:H58" si="1">F54+G54</f>
+        <f t="shared" ref="H54:H58" si="0">F54+G54</f>
         <v>0</v>
       </c>
-      <c r="I54" s="145">
-        <f>I53-H54</f>
-        <v>20202426</v>
-      </c>
+      <c r="I54" s="145"/>
       <c r="J54" s="212"/>
       <c r="K54" s="141"/>
       <c r="N54" s="24"/>
@@ -4034,13 +3816,10 @@
       <c r="F55" s="144"/>
       <c r="G55" s="144"/>
       <c r="H55" s="144">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I55" s="145">
-        <f>I54-H55</f>
-        <v>20202426</v>
-      </c>
+      <c r="I55" s="145"/>
       <c r="J55" s="212"/>
       <c r="K55" s="141"/>
       <c r="N55" s="24"/>
@@ -4060,13 +3839,10 @@
       <c r="F56" s="144"/>
       <c r="G56" s="144"/>
       <c r="H56" s="144">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I56" s="145">
-        <f t="shared" ref="I56:I58" si="2">I55-H56</f>
-        <v>20202426</v>
-      </c>
+      <c r="I56" s="145"/>
       <c r="J56" s="212"/>
       <c r="K56" s="141"/>
       <c r="N56" s="24"/>
@@ -4086,13 +3862,10 @@
       <c r="F57" s="144"/>
       <c r="G57" s="144"/>
       <c r="H57" s="144">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I57" s="145">
-        <f t="shared" si="2"/>
-        <v>20202426</v>
-      </c>
+      <c r="I57" s="145"/>
       <c r="J57" s="212"/>
       <c r="K57" s="141"/>
       <c r="N57" s="24"/>
@@ -4112,13 +3885,10 @@
       <c r="F58" s="144"/>
       <c r="G58" s="144"/>
       <c r="H58" s="144">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I58" s="145">
-        <f t="shared" si="2"/>
-        <v>20202426</v>
-      </c>
+      <c r="I58" s="145"/>
       <c r="J58" s="212"/>
       <c r="K58" s="141"/>
       <c r="N58" s="24"/>
@@ -4130,11 +3900,11 @@
     <row r="59" spans="1:73" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="135"/>
       <c r="B59" s="184"/>
-      <c r="C59" s="266" t="s">
+      <c r="C59" s="300" t="s">
         <v>71</v>
       </c>
-      <c r="D59" s="267"/>
-      <c r="E59" s="268"/>
+      <c r="D59" s="301"/>
+      <c r="E59" s="302"/>
       <c r="F59" s="146">
         <f>SUM(F53:F58)</f>
         <v>0</v>
@@ -4159,22 +3929,19 @@
     <row r="60" spans="1:73" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="135"/>
       <c r="B60" s="184"/>
-      <c r="C60" s="266" t="s">
+      <c r="C60" s="300" t="s">
         <v>72</v>
       </c>
-      <c r="D60" s="267"/>
-      <c r="E60" s="268"/>
-      <c r="F60" s="144">
-        <f>K15</f>
-        <v>20202426</v>
-      </c>
+      <c r="D60" s="301"/>
+      <c r="E60" s="302"/>
+      <c r="F60" s="144"/>
       <c r="G60" s="144">
         <f>K16</f>
         <v>0</v>
       </c>
       <c r="H60" s="144">
         <f>SUM(F60:G60)</f>
-        <v>20202426</v>
+        <v>0</v>
       </c>
       <c r="I60" s="145"/>
       <c r="J60" s="212"/>
@@ -4188,14 +3955,14 @@
     <row r="61" spans="1:73" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="242"/>
       <c r="B61" s="239"/>
-      <c r="C61" s="266" t="s">
+      <c r="C61" s="300" t="s">
         <v>73</v>
       </c>
-      <c r="D61" s="267"/>
-      <c r="E61" s="268"/>
+      <c r="D61" s="301"/>
+      <c r="E61" s="302"/>
       <c r="F61" s="146">
         <f>F60-F59</f>
-        <v>20202426</v>
+        <v>0</v>
       </c>
       <c r="G61" s="146">
         <f>G60-G59</f>
@@ -4203,7 +3970,7 @@
       </c>
       <c r="H61" s="146">
         <f>H60-H59</f>
-        <v>20202426</v>
+        <v>0</v>
       </c>
       <c r="I61" s="145"/>
       <c r="J61" s="243"/>
@@ -4250,19 +4017,19 @@
       </c>
     </row>
     <row r="64" spans="1:73" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="257" t="s">
+      <c r="A64" s="321" t="s">
         <v>74</v>
       </c>
-      <c r="B64" s="257"/>
-      <c r="C64" s="257"/>
-      <c r="D64" s="257"/>
-      <c r="E64" s="257"/>
-      <c r="F64" s="257"/>
-      <c r="G64" s="257"/>
-      <c r="H64" s="257"/>
-      <c r="I64" s="257"/>
-      <c r="J64" s="257"/>
-      <c r="K64" s="257"/>
+      <c r="B64" s="321"/>
+      <c r="C64" s="321"/>
+      <c r="D64" s="321"/>
+      <c r="E64" s="321"/>
+      <c r="F64" s="321"/>
+      <c r="G64" s="321"/>
+      <c r="H64" s="321"/>
+      <c r="I64" s="321"/>
+      <c r="J64" s="321"/>
+      <c r="K64" s="321"/>
       <c r="Z64" s="6"/>
       <c r="BU64" s="84">
         <v>44956</v>
@@ -4287,19 +4054,19 @@
       </c>
     </row>
     <row r="66" spans="1:73" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="301" t="s">
+      <c r="A66" s="305" t="s">
         <v>75</v>
       </c>
-      <c r="B66" s="302"/>
-      <c r="C66" s="302"/>
-      <c r="D66" s="302"/>
-      <c r="E66" s="302"/>
-      <c r="F66" s="302"/>
-      <c r="G66" s="302"/>
-      <c r="H66" s="302"/>
-      <c r="I66" s="302"/>
-      <c r="J66" s="302"/>
-      <c r="K66" s="303"/>
+      <c r="B66" s="306"/>
+      <c r="C66" s="306"/>
+      <c r="D66" s="306"/>
+      <c r="E66" s="306"/>
+      <c r="F66" s="306"/>
+      <c r="G66" s="306"/>
+      <c r="H66" s="306"/>
+      <c r="I66" s="306"/>
+      <c r="J66" s="306"/>
+      <c r="K66" s="307"/>
       <c r="N66" s="7"/>
       <c r="Z66" s="6"/>
       <c r="BU66" s="84">
@@ -4315,7 +4082,7 @@
       </c>
       <c r="E67" s="184"/>
       <c r="F67" s="219" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="G67" s="220"/>
       <c r="H67" s="220"/>
@@ -4329,19 +4096,19 @@
       </c>
     </row>
     <row r="68" spans="1:73" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="261" t="s">
+      <c r="A68" s="341" t="s">
         <v>78</v>
       </c>
-      <c r="B68" s="262"/>
-      <c r="C68" s="262"/>
-      <c r="D68" s="262"/>
-      <c r="E68" s="262"/>
-      <c r="F68" s="262"/>
-      <c r="G68" s="262"/>
-      <c r="H68" s="262"/>
-      <c r="I68" s="262"/>
-      <c r="J68" s="262"/>
-      <c r="K68" s="263"/>
+      <c r="B68" s="342"/>
+      <c r="C68" s="342"/>
+      <c r="D68" s="342"/>
+      <c r="E68" s="342"/>
+      <c r="F68" s="342"/>
+      <c r="G68" s="342"/>
+      <c r="H68" s="342"/>
+      <c r="I68" s="342"/>
+      <c r="J68" s="342"/>
+      <c r="K68" s="343"/>
       <c r="N68" s="7"/>
       <c r="Z68" s="6"/>
       <c r="BU68" s="84">
@@ -4367,17 +4134,17 @@
       </c>
     </row>
     <row r="70" spans="1:73" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="261" t="s">
+      <c r="A70" s="341" t="s">
         <v>79</v>
       </c>
-      <c r="B70" s="262"/>
-      <c r="C70" s="262"/>
-      <c r="D70" s="262"/>
-      <c r="E70" s="262"/>
-      <c r="F70" s="262"/>
-      <c r="G70" s="262"/>
-      <c r="H70" s="262"/>
-      <c r="I70" s="262"/>
+      <c r="B70" s="342"/>
+      <c r="C70" s="342"/>
+      <c r="D70" s="342"/>
+      <c r="E70" s="342"/>
+      <c r="F70" s="342"/>
+      <c r="G70" s="342"/>
+      <c r="H70" s="342"/>
+      <c r="I70" s="342"/>
       <c r="J70" s="221"/>
       <c r="K70" s="181"/>
       <c r="N70" s="7"/>
@@ -4391,7 +4158,7 @@
       <c r="B71" s="221"/>
       <c r="C71" s="221"/>
       <c r="D71" s="219" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E71" s="184"/>
       <c r="F71" s="219" t="s">
@@ -4409,19 +4176,19 @@
       </c>
     </row>
     <row r="72" spans="1:73" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="329" t="s">
+      <c r="A72" s="261" t="s">
         <v>80</v>
       </c>
-      <c r="B72" s="330"/>
-      <c r="C72" s="330"/>
-      <c r="D72" s="330"/>
-      <c r="E72" s="330"/>
-      <c r="F72" s="330"/>
-      <c r="G72" s="330"/>
-      <c r="H72" s="330"/>
-      <c r="I72" s="330"/>
-      <c r="J72" s="330"/>
-      <c r="K72" s="331"/>
+      <c r="B72" s="262"/>
+      <c r="C72" s="262"/>
+      <c r="D72" s="262"/>
+      <c r="E72" s="262"/>
+      <c r="F72" s="262"/>
+      <c r="G72" s="262"/>
+      <c r="H72" s="262"/>
+      <c r="I72" s="262"/>
+      <c r="J72" s="262"/>
+      <c r="K72" s="263"/>
       <c r="N72" s="7"/>
       <c r="Z72" s="6"/>
       <c r="BU72" s="84">
@@ -4447,19 +4214,19 @@
       </c>
     </row>
     <row r="74" spans="1:73" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="257" t="s">
+      <c r="A74" s="321" t="s">
         <v>81</v>
       </c>
-      <c r="B74" s="257"/>
-      <c r="C74" s="257"/>
-      <c r="D74" s="257"/>
-      <c r="E74" s="257"/>
-      <c r="F74" s="257"/>
-      <c r="G74" s="257"/>
-      <c r="H74" s="257"/>
-      <c r="I74" s="257"/>
-      <c r="J74" s="257"/>
-      <c r="K74" s="257"/>
+      <c r="B74" s="321"/>
+      <c r="C74" s="321"/>
+      <c r="D74" s="321"/>
+      <c r="E74" s="321"/>
+      <c r="F74" s="321"/>
+      <c r="G74" s="321"/>
+      <c r="H74" s="321"/>
+      <c r="I74" s="321"/>
+      <c r="J74" s="321"/>
+      <c r="K74" s="321"/>
       <c r="Z74" s="6"/>
       <c r="BU74" s="84">
         <v>44966</v>
@@ -4486,20 +4253,20 @@
     <row r="76" spans="1:73" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A76" s="93"/>
       <c r="B76" s="223"/>
-      <c r="C76" s="314" t="s">
+      <c r="C76" s="290" t="s">
         <v>82</v>
       </c>
-      <c r="D76" s="315"/>
-      <c r="E76" s="155">
+      <c r="D76" s="291"/>
+      <c r="E76" s="155" t="e">
         <f>H59/H60</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="F76" s="184"/>
       <c r="G76" s="223"/>
-      <c r="H76" s="314" t="s">
+      <c r="H76" s="290" t="s">
         <v>83</v>
       </c>
-      <c r="I76" s="315"/>
+      <c r="I76" s="291"/>
       <c r="J76" s="155">
         <f>1/180</f>
         <v>5.5555555555555558E-3</v>
@@ -4547,17 +4314,17 @@
     </row>
     <row r="79" spans="1:73" s="17" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A79" s="228"/>
-      <c r="B79" s="294" t="s">
+      <c r="B79" s="309" t="s">
         <v>84</v>
       </c>
-      <c r="C79" s="295"/>
-      <c r="D79" s="296"/>
-      <c r="E79" s="294" t="s">
+      <c r="C79" s="310"/>
+      <c r="D79" s="311"/>
+      <c r="E79" s="309" t="s">
         <v>85</v>
       </c>
-      <c r="F79" s="295"/>
-      <c r="G79" s="295"/>
-      <c r="H79" s="296"/>
+      <c r="F79" s="310"/>
+      <c r="G79" s="310"/>
+      <c r="H79" s="311"/>
       <c r="I79" s="159" t="s">
         <v>86</v>
       </c>
@@ -4572,48 +4339,32 @@
     </row>
     <row r="80" spans="1:73" s="17" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="228"/>
-      <c r="B80" s="258" t="s">
-        <v>208</v>
-      </c>
+      <c r="B80" s="258"/>
       <c r="C80" s="259"/>
       <c r="D80" s="260"/>
-      <c r="E80" s="177" t="s">
-        <v>212</v>
-      </c>
+      <c r="E80" s="177"/>
       <c r="F80" s="178"/>
       <c r="G80" s="178"/>
       <c r="H80" s="179"/>
-      <c r="I80" s="252" t="s">
-        <v>216</v>
-      </c>
-      <c r="J80" s="161">
-        <v>1</v>
-      </c>
+      <c r="I80" s="252"/>
+      <c r="J80" s="161"/>
       <c r="K80" s="158"/>
       <c r="L80" s="2"/>
       <c r="BU80" s="84">
         <v>44971</v>
       </c>
     </row>
-    <row r="81" spans="1:73" s="17" customFormat="1" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:73" s="17" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A81" s="228"/>
-      <c r="B81" s="258" t="s">
-        <v>209</v>
-      </c>
+      <c r="B81" s="258"/>
       <c r="C81" s="259"/>
       <c r="D81" s="260"/>
-      <c r="E81" s="258" t="s">
-        <v>213</v>
-      </c>
+      <c r="E81" s="258"/>
       <c r="F81" s="259"/>
       <c r="G81" s="259"/>
       <c r="H81" s="260"/>
-      <c r="I81" s="160" t="s">
-        <v>217</v>
-      </c>
-      <c r="J81" s="161">
-        <v>1</v>
-      </c>
+      <c r="I81" s="160"/>
+      <c r="J81" s="161"/>
       <c r="K81" s="158"/>
       <c r="L81" s="2"/>
       <c r="BU81" s="84">
@@ -4622,14 +4373,10 @@
     </row>
     <row r="82" spans="1:73" s="17" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A82" s="228"/>
-      <c r="B82" s="258" t="s">
-        <v>210</v>
-      </c>
+      <c r="B82" s="258"/>
       <c r="C82" s="259"/>
       <c r="D82" s="260"/>
-      <c r="E82" s="258" t="s">
-        <v>214</v>
-      </c>
+      <c r="E82" s="258"/>
       <c r="F82" s="259"/>
       <c r="G82" s="259"/>
       <c r="H82" s="260"/>
@@ -4643,14 +4390,10 @@
     </row>
     <row r="83" spans="1:73" s="17" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A83" s="228"/>
-      <c r="B83" s="258" t="s">
-        <v>211</v>
-      </c>
+      <c r="B83" s="258"/>
       <c r="C83" s="259"/>
       <c r="D83" s="260"/>
-      <c r="E83" s="258" t="s">
-        <v>215</v>
-      </c>
+      <c r="E83" s="258"/>
       <c r="F83" s="259"/>
       <c r="G83" s="259"/>
       <c r="H83" s="260"/>
@@ -4664,9 +4407,7 @@
     </row>
     <row r="84" spans="1:73" s="17" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A84" s="228"/>
-      <c r="B84" s="258" t="s">
-        <v>218</v>
-      </c>
+      <c r="B84" s="258"/>
       <c r="C84" s="259"/>
       <c r="D84" s="260"/>
       <c r="E84" s="258"/>
@@ -5227,55 +4968,55 @@
       </c>
     </row>
     <row r="119" spans="1:73" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="288" t="s">
+      <c r="A119" s="328" t="s">
         <v>88</v>
       </c>
-      <c r="B119" s="289"/>
-      <c r="C119" s="289"/>
-      <c r="D119" s="289"/>
-      <c r="E119" s="289"/>
-      <c r="F119" s="289"/>
-      <c r="G119" s="289"/>
-      <c r="H119" s="289"/>
-      <c r="I119" s="289"/>
-      <c r="J119" s="289"/>
-      <c r="K119" s="290"/>
+      <c r="B119" s="329"/>
+      <c r="C119" s="329"/>
+      <c r="D119" s="329"/>
+      <c r="E119" s="329"/>
+      <c r="F119" s="329"/>
+      <c r="G119" s="329"/>
+      <c r="H119" s="329"/>
+      <c r="I119" s="329"/>
+      <c r="J119" s="329"/>
+      <c r="K119" s="330"/>
       <c r="Z119" s="6"/>
       <c r="BU119" s="84">
         <v>45010</v>
       </c>
     </row>
     <row r="120" spans="1:73" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="291"/>
-      <c r="B120" s="292"/>
-      <c r="C120" s="292"/>
-      <c r="D120" s="292"/>
-      <c r="E120" s="292"/>
-      <c r="F120" s="292"/>
-      <c r="G120" s="292"/>
-      <c r="H120" s="292"/>
-      <c r="I120" s="292"/>
-      <c r="J120" s="292"/>
-      <c r="K120" s="293"/>
+      <c r="A120" s="331"/>
+      <c r="B120" s="332"/>
+      <c r="C120" s="332"/>
+      <c r="D120" s="332"/>
+      <c r="E120" s="332"/>
+      <c r="F120" s="332"/>
+      <c r="G120" s="332"/>
+      <c r="H120" s="332"/>
+      <c r="I120" s="332"/>
+      <c r="J120" s="332"/>
+      <c r="K120" s="333"/>
       <c r="Z120" s="6"/>
       <c r="BU120" s="84">
         <v>45011</v>
       </c>
     </row>
     <row r="121" spans="1:73" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A121" s="257" t="s">
+      <c r="A121" s="321" t="s">
         <v>89</v>
       </c>
-      <c r="B121" s="257"/>
-      <c r="C121" s="257"/>
-      <c r="D121" s="257"/>
-      <c r="E121" s="257"/>
-      <c r="F121" s="257"/>
-      <c r="G121" s="257"/>
-      <c r="H121" s="257"/>
-      <c r="I121" s="257"/>
-      <c r="J121" s="257"/>
-      <c r="K121" s="257"/>
+      <c r="B121" s="321"/>
+      <c r="C121" s="321"/>
+      <c r="D121" s="321"/>
+      <c r="E121" s="321"/>
+      <c r="F121" s="321"/>
+      <c r="G121" s="321"/>
+      <c r="H121" s="321"/>
+      <c r="I121" s="321"/>
+      <c r="J121" s="321"/>
+      <c r="K121" s="321"/>
       <c r="N121" s="2"/>
       <c r="BU121" s="84">
         <v>45012</v>
@@ -5304,17 +5045,15 @@
       <c r="A123" s="166" t="s">
         <v>90</v>
       </c>
-      <c r="B123" s="269"/>
-      <c r="C123" s="269"/>
+      <c r="B123" s="276"/>
+      <c r="C123" s="276"/>
       <c r="E123" s="184"/>
       <c r="F123" s="184"/>
       <c r="G123" s="230" t="s">
         <v>92</v>
       </c>
-      <c r="H123" s="269">
-        <v>1000191780</v>
-      </c>
-      <c r="I123" s="269"/>
+      <c r="H123" s="276"/>
+      <c r="I123" s="276"/>
       <c r="J123" s="227"/>
       <c r="K123" s="158"/>
       <c r="N123" s="2"/>
@@ -5356,17 +5095,17 @@
       </c>
     </row>
     <row r="126" spans="1:73" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A126" s="342" t="s">
+      <c r="A126" s="274" t="s">
         <v>93</v>
       </c>
-      <c r="B126" s="343"/>
-      <c r="C126" s="343"/>
-      <c r="D126" s="343"/>
-      <c r="E126" s="343"/>
-      <c r="F126" s="343"/>
-      <c r="G126" s="343"/>
-      <c r="H126" s="343"/>
-      <c r="I126" s="343"/>
+      <c r="B126" s="275"/>
+      <c r="C126" s="275"/>
+      <c r="D126" s="275"/>
+      <c r="E126" s="275"/>
+      <c r="F126" s="275"/>
+      <c r="G126" s="275"/>
+      <c r="H126" s="275"/>
+      <c r="I126" s="275"/>
       <c r="J126" s="227"/>
       <c r="K126" s="158"/>
       <c r="Z126" s="6"/>
@@ -5375,15 +5114,15 @@
       </c>
     </row>
     <row r="127" spans="1:73" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A127" s="342"/>
-      <c r="B127" s="343"/>
-      <c r="C127" s="343"/>
-      <c r="D127" s="343"/>
-      <c r="E127" s="343"/>
-      <c r="F127" s="343"/>
-      <c r="G127" s="343"/>
-      <c r="H127" s="343"/>
-      <c r="I127" s="343"/>
+      <c r="A127" s="274"/>
+      <c r="B127" s="275"/>
+      <c r="C127" s="275"/>
+      <c r="D127" s="275"/>
+      <c r="E127" s="275"/>
+      <c r="F127" s="275"/>
+      <c r="G127" s="275"/>
+      <c r="H127" s="275"/>
+      <c r="I127" s="275"/>
       <c r="J127" s="233"/>
       <c r="K127" s="168"/>
       <c r="Z127" s="6"/>
@@ -5447,17 +5186,17 @@
       </c>
     </row>
     <row r="131" spans="1:73" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A131" s="340" t="s">
+      <c r="A131" s="272" t="s">
         <v>95</v>
       </c>
-      <c r="B131" s="341"/>
-      <c r="C131" s="341"/>
-      <c r="D131" s="341"/>
-      <c r="E131" s="341"/>
-      <c r="F131" s="341"/>
-      <c r="G131" s="341"/>
-      <c r="H131" s="341"/>
-      <c r="I131" s="341"/>
+      <c r="B131" s="273"/>
+      <c r="C131" s="273"/>
+      <c r="D131" s="273"/>
+      <c r="E131" s="273"/>
+      <c r="F131" s="273"/>
+      <c r="G131" s="273"/>
+      <c r="H131" s="273"/>
+      <c r="I131" s="273"/>
       <c r="J131" s="236"/>
       <c r="K131" s="171"/>
       <c r="Z131" s="6"/>
@@ -5522,17 +5261,15 @@
       <c r="A135" s="172" t="s">
         <v>97</v>
       </c>
-      <c r="B135" s="269"/>
-      <c r="C135" s="269"/>
+      <c r="B135" s="276"/>
+      <c r="C135" s="276"/>
       <c r="D135" s="191"/>
       <c r="E135" s="230" t="s">
         <v>98</v>
       </c>
       <c r="F135" s="191"/>
-      <c r="G135" s="300">
-        <v>46079</v>
-      </c>
-      <c r="H135" s="300"/>
+      <c r="G135" s="308"/>
+      <c r="H135" s="308"/>
       <c r="I135" s="227"/>
       <c r="J135" s="227"/>
       <c r="K135" s="158"/>
@@ -5545,10 +5282,8 @@
       <c r="A136" s="172" t="s">
         <v>99</v>
       </c>
-      <c r="B136" s="270">
-        <v>98663128</v>
-      </c>
-      <c r="C136" s="270"/>
+      <c r="B136" s="287"/>
+      <c r="C136" s="287"/>
       <c r="D136" s="191"/>
       <c r="E136" s="230"/>
       <c r="F136" s="191"/>
@@ -5591,49 +5326,49 @@
       <c r="BU138" s="84"/>
     </row>
     <row r="139" spans="1:73" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A139" s="336" t="s">
+      <c r="A139" s="268" t="s">
         <v>100</v>
       </c>
-      <c r="B139" s="337"/>
-      <c r="C139" s="337"/>
-      <c r="D139" s="337"/>
-      <c r="E139" s="337"/>
-      <c r="F139" s="337"/>
-      <c r="G139" s="337"/>
-      <c r="H139" s="337"/>
-      <c r="I139" s="337"/>
-      <c r="J139" s="337"/>
-      <c r="K139" s="338"/>
+      <c r="B139" s="269"/>
+      <c r="C139" s="269"/>
+      <c r="D139" s="269"/>
+      <c r="E139" s="269"/>
+      <c r="F139" s="269"/>
+      <c r="G139" s="269"/>
+      <c r="H139" s="269"/>
+      <c r="I139" s="269"/>
+      <c r="J139" s="269"/>
+      <c r="K139" s="270"/>
       <c r="Z139" s="6"/>
       <c r="BU139" s="84"/>
     </row>
     <row r="140" spans="1:73" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A140" s="339"/>
-      <c r="B140" s="337"/>
-      <c r="C140" s="337"/>
-      <c r="D140" s="337"/>
-      <c r="E140" s="337"/>
-      <c r="F140" s="337"/>
-      <c r="G140" s="337"/>
-      <c r="H140" s="337"/>
-      <c r="I140" s="337"/>
-      <c r="J140" s="337"/>
-      <c r="K140" s="338"/>
+      <c r="A140" s="271"/>
+      <c r="B140" s="269"/>
+      <c r="C140" s="269"/>
+      <c r="D140" s="269"/>
+      <c r="E140" s="269"/>
+      <c r="F140" s="269"/>
+      <c r="G140" s="269"/>
+      <c r="H140" s="269"/>
+      <c r="I140" s="269"/>
+      <c r="J140" s="269"/>
+      <c r="K140" s="270"/>
       <c r="Z140" s="6"/>
       <c r="BU140" s="84"/>
     </row>
     <row r="141" spans="1:73" ht="1.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A141" s="339"/>
-      <c r="B141" s="337"/>
-      <c r="C141" s="337"/>
-      <c r="D141" s="337"/>
-      <c r="E141" s="337"/>
-      <c r="F141" s="337"/>
-      <c r="G141" s="337"/>
-      <c r="H141" s="337"/>
-      <c r="I141" s="337"/>
-      <c r="J141" s="337"/>
-      <c r="K141" s="338"/>
+      <c r="A141" s="271"/>
+      <c r="B141" s="269"/>
+      <c r="C141" s="269"/>
+      <c r="D141" s="269"/>
+      <c r="E141" s="269"/>
+      <c r="F141" s="269"/>
+      <c r="G141" s="269"/>
+      <c r="H141" s="269"/>
+      <c r="I141" s="269"/>
+      <c r="J141" s="269"/>
+      <c r="K141" s="270"/>
       <c r="Z141" s="6"/>
       <c r="BU141" s="84"/>
     </row>
@@ -5647,10 +5382,10 @@
       <c r="G142" s="199"/>
       <c r="H142" s="199"/>
       <c r="I142" s="227"/>
-      <c r="J142" s="332" t="s">
+      <c r="J142" s="264" t="s">
         <v>101</v>
       </c>
-      <c r="K142" s="333"/>
+      <c r="K142" s="265"/>
       <c r="Z142" s="6"/>
       <c r="BU142" s="84"/>
     </row>
@@ -5664,8 +5399,8 @@
       <c r="G143" s="176"/>
       <c r="H143" s="176"/>
       <c r="I143" s="176"/>
-      <c r="J143" s="334"/>
-      <c r="K143" s="335"/>
+      <c r="J143" s="266"/>
+      <c r="K143" s="267"/>
       <c r="Z143" s="6"/>
       <c r="BU143" s="84">
         <v>45027</v>
@@ -13421,6 +13156,127 @@
     <protectedRange sqref="A122:C122" name="Rango1_1_1"/>
   </protectedRanges>
   <mergeCells count="145">
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="A64:K64"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B82:D82"/>
+    <mergeCell ref="B84:D84"/>
+    <mergeCell ref="E105:H105"/>
+    <mergeCell ref="A68:K68"/>
+    <mergeCell ref="B102:D102"/>
+    <mergeCell ref="B89:D89"/>
+    <mergeCell ref="E101:H101"/>
+    <mergeCell ref="E102:H102"/>
+    <mergeCell ref="B115:D115"/>
+    <mergeCell ref="B116:D116"/>
+    <mergeCell ref="B117:D117"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="E109:H109"/>
+    <mergeCell ref="E110:H110"/>
+    <mergeCell ref="E98:H98"/>
+    <mergeCell ref="E99:H99"/>
+    <mergeCell ref="E100:H100"/>
+    <mergeCell ref="B113:D113"/>
+    <mergeCell ref="B114:D114"/>
+    <mergeCell ref="C60:E60"/>
+    <mergeCell ref="A70:I70"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="B135:C135"/>
+    <mergeCell ref="B136:C136"/>
+    <mergeCell ref="B10:K13"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="A25:K25"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="A74:K74"/>
+    <mergeCell ref="A121:K121"/>
+    <mergeCell ref="A119:K120"/>
+    <mergeCell ref="E79:H79"/>
+    <mergeCell ref="E81:H81"/>
+    <mergeCell ref="E82:H82"/>
+    <mergeCell ref="E83:H83"/>
+    <mergeCell ref="E84:H84"/>
+    <mergeCell ref="E85:H85"/>
+    <mergeCell ref="E86:H86"/>
+    <mergeCell ref="E87:H87"/>
+    <mergeCell ref="B112:D112"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="B111:D111"/>
+    <mergeCell ref="B104:D104"/>
+    <mergeCell ref="G135:H135"/>
+    <mergeCell ref="E115:H115"/>
+    <mergeCell ref="E116:H116"/>
+    <mergeCell ref="E117:H117"/>
+    <mergeCell ref="B79:D79"/>
+    <mergeCell ref="B91:D91"/>
+    <mergeCell ref="B92:D92"/>
+    <mergeCell ref="B93:D93"/>
+    <mergeCell ref="B94:D94"/>
+    <mergeCell ref="B95:D95"/>
+    <mergeCell ref="B96:D96"/>
+    <mergeCell ref="B97:D97"/>
+    <mergeCell ref="B98:D98"/>
+    <mergeCell ref="B99:D99"/>
+    <mergeCell ref="B100:D100"/>
+    <mergeCell ref="B101:D101"/>
+    <mergeCell ref="B83:D83"/>
+    <mergeCell ref="E88:H88"/>
+    <mergeCell ref="E89:H89"/>
+    <mergeCell ref="B86:D86"/>
+    <mergeCell ref="E103:H103"/>
+    <mergeCell ref="B103:D103"/>
+    <mergeCell ref="B80:D80"/>
+    <mergeCell ref="B81:D81"/>
+    <mergeCell ref="E113:H113"/>
+    <mergeCell ref="E114:H114"/>
+    <mergeCell ref="E97:H97"/>
+    <mergeCell ref="B106:D106"/>
+    <mergeCell ref="B107:D107"/>
+    <mergeCell ref="B108:D108"/>
+    <mergeCell ref="E104:H104"/>
+    <mergeCell ref="A66:K66"/>
+    <mergeCell ref="E106:H106"/>
+    <mergeCell ref="B105:D105"/>
+    <mergeCell ref="E107:H107"/>
+    <mergeCell ref="E108:H108"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="C8:E8"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="H76:I76"/>
+    <mergeCell ref="C76:D76"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="C31:I31"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="D40:E40"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="B15:B16"/>
     <mergeCell ref="B109:D109"/>
@@ -13445,129 +13301,8 @@
     <mergeCell ref="E96:H96"/>
     <mergeCell ref="E111:H111"/>
     <mergeCell ref="E112:H112"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="H76:I76"/>
-    <mergeCell ref="C76:D76"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="G29:I29"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="C31:I31"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="C61:E61"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="E113:H113"/>
-    <mergeCell ref="E114:H114"/>
-    <mergeCell ref="E97:H97"/>
-    <mergeCell ref="B106:D106"/>
-    <mergeCell ref="B107:D107"/>
-    <mergeCell ref="B108:D108"/>
-    <mergeCell ref="E104:H104"/>
-    <mergeCell ref="A66:K66"/>
-    <mergeCell ref="E106:H106"/>
-    <mergeCell ref="B105:D105"/>
-    <mergeCell ref="E107:H107"/>
-    <mergeCell ref="E108:H108"/>
-    <mergeCell ref="G135:H135"/>
-    <mergeCell ref="E115:H115"/>
-    <mergeCell ref="E116:H116"/>
-    <mergeCell ref="E117:H117"/>
-    <mergeCell ref="B79:D79"/>
-    <mergeCell ref="B91:D91"/>
-    <mergeCell ref="B92:D92"/>
-    <mergeCell ref="B93:D93"/>
-    <mergeCell ref="B94:D94"/>
-    <mergeCell ref="B95:D95"/>
-    <mergeCell ref="B96:D96"/>
-    <mergeCell ref="B97:D97"/>
-    <mergeCell ref="B98:D98"/>
-    <mergeCell ref="B99:D99"/>
-    <mergeCell ref="B100:D100"/>
-    <mergeCell ref="B101:D101"/>
-    <mergeCell ref="B83:D83"/>
-    <mergeCell ref="E88:H88"/>
-    <mergeCell ref="E89:H89"/>
-    <mergeCell ref="B86:D86"/>
-    <mergeCell ref="E103:H103"/>
-    <mergeCell ref="B103:D103"/>
-    <mergeCell ref="B80:D80"/>
-    <mergeCell ref="B81:D81"/>
-    <mergeCell ref="B135:C135"/>
-    <mergeCell ref="B136:C136"/>
-    <mergeCell ref="B10:K13"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="G23:J23"/>
-    <mergeCell ref="A25:K25"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="A74:K74"/>
-    <mergeCell ref="A121:K121"/>
-    <mergeCell ref="A119:K120"/>
-    <mergeCell ref="E79:H79"/>
-    <mergeCell ref="E81:H81"/>
-    <mergeCell ref="E82:H82"/>
-    <mergeCell ref="E83:H83"/>
-    <mergeCell ref="E84:H84"/>
-    <mergeCell ref="E85:H85"/>
-    <mergeCell ref="E86:H86"/>
-    <mergeCell ref="E87:H87"/>
-    <mergeCell ref="B112:D112"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="B111:D111"/>
-    <mergeCell ref="B104:D104"/>
-    <mergeCell ref="B115:D115"/>
-    <mergeCell ref="B116:D116"/>
-    <mergeCell ref="B117:D117"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="E109:H109"/>
-    <mergeCell ref="E110:H110"/>
-    <mergeCell ref="E98:H98"/>
-    <mergeCell ref="E99:H99"/>
-    <mergeCell ref="E100:H100"/>
-    <mergeCell ref="B113:D113"/>
-    <mergeCell ref="B114:D114"/>
-    <mergeCell ref="C60:E60"/>
-    <mergeCell ref="A70:I70"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="C59:E59"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="A64:K64"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B82:D82"/>
-    <mergeCell ref="B84:D84"/>
-    <mergeCell ref="E105:H105"/>
-    <mergeCell ref="A68:K68"/>
-    <mergeCell ref="B102:D102"/>
-    <mergeCell ref="B89:D89"/>
-    <mergeCell ref="E101:H101"/>
-    <mergeCell ref="E102:H102"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="9">
+  <dataValidations count="9">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F63 G45:G49" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>$AC$2:$AC$5</formula1>
     </dataValidation>
@@ -13596,17 +13331,14 @@
       <formula1>$BU$37:$BU$767</formula1>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink ref="I80" r:id="rId1" xr:uid="{55020FA7-40C9-441D-8723-0F48B6B4247A}"/>
-  </hyperlinks>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="52" fitToHeight="0" orientation="landscape" r:id="rId2"/>
+  <pageSetup scale="52" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <rowBreaks count="2" manualBreakCount="2">
     <brk id="24" max="10" man="1"/>
     <brk id="120" max="10" man="1"/>
   </rowBreaks>
-  <drawing r:id="rId3"/>
-  <legacyDrawing r:id="rId4"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -14318,6 +14050,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="54909ea9-b8a6-49fb-80e9-be6d07efd491">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="0114b50f-9d75-4745-893c-845a73c5ba4a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006098FC569B2E844387057BC377073F07" ma:contentTypeVersion="14" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a1e562420dc294ed62ccd2f77b457a64">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="54909ea9-b8a6-49fb-80e9-be6d07efd491" xmlns:ns3="0114b50f-9d75-4745-893c-845a73c5ba4a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b191f6e8884aab5c11f83754b5d6b2f9" ns2:_="" ns3:_="">
     <xsd:import namespace="54909ea9-b8a6-49fb-80e9-be6d07efd491"/>
@@ -14548,17 +14291,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="54909ea9-b8a6-49fb-80e9-be6d07efd491">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="0114b50f-9d75-4745-893c-845a73c5ba4a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -14569,6 +14301,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DBEFA19-BD66-4F6E-9F31-A9D8BF2EC2BB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="54909ea9-b8a6-49fb-80e9-be6d07efd491"/>
+    <ds:schemaRef ds:uri="0114b50f-9d75-4745-893c-845a73c5ba4a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F6CD79D-EAE6-4C11-B69C-B1C11900EC25}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -14587,17 +14330,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DBEFA19-BD66-4F6E-9F31-A9D8BF2EC2BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="54909ea9-b8a6-49fb-80e9-be6d07efd491"/>
-    <ds:schemaRef ds:uri="0114b50f-9d75-4745-893c-845a73c5ba4a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{119A69A5-E964-441A-AB6D-5D848257286A}">
   <ds:schemaRefs>

</xml_diff>